<commit_message>
test the rachford rice algorithm for the whole dataset and test the results. Also some adjustments were made to the datasets.
</commit_message>
<xml_diff>
--- a/UnifacDortmund/Experimental_Data/data/comps_MW.xlsx
+++ b/UnifacDortmund/Experimental_Data/data/comps_MW.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27928"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Juan\Maestría\Code\oleosim\UnifacDortmund\Experimental_Data\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Juan\proyectos_personales\Maestría\Materias\Tesis\oleosim\UnifacDortmund\Experimental_Data\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D84A7F4-17B6-4921-B01A-DE0D8D5752CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2744DE7-B3C7-4095-8A1D-FFEC06D7726E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2340" yWindow="2340" windowWidth="21570" windowHeight="11280" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="20">
   <si>
     <t>Ref</t>
   </si>
@@ -139,9 +139,6 @@
       <numFmt numFmtId="164" formatCode="#,##0;[Red]\-#,##0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="#,##0;[Red]\-#,##0"/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="165" formatCode="#,##0.000;[Red]\-#,##0.000"/>
     </dxf>
     <dxf>
@@ -165,6 +162,9 @@
     <dxf>
       <numFmt numFmtId="164" formatCode="#,##0;[Red]\-#,##0"/>
     </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="#,##0;[Red]\-#,##0"/>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -179,20 +179,20 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Frame0" displayName="Frame0" ref="A1:K96" totalsRowShown="0">
-  <autoFilter ref="A1:K96" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Frame0" displayName="Frame0" ref="A1:K95" totalsRowShown="0">
+  <autoFilter ref="A1:K95" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="11">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Ref" dataDxfId="9"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Sub Ref"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Type Alcohol" dataDxfId="0"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="MW_FAME/FAEE" dataDxfId="8"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="MW_Glycerol" dataDxfId="7"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="MW_Alcohol" dataDxfId="6"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="MW_Oil" dataDxfId="5"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="MW_DAG" dataDxfId="4"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="MW_MAG" dataDxfId="3"/>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="MW_FA" dataDxfId="2"/>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="MW_H2O" dataDxfId="1"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Type Alcohol" dataDxfId="8"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="MW_FAME/FAEE" dataDxfId="7"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="MW_Glycerol" dataDxfId="6"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="MW_Alcohol" dataDxfId="5"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="MW_Oil" dataDxfId="4"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="MW_DAG" dataDxfId="3"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="MW_MAG" dataDxfId="2"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="MW_FA" dataDxfId="1"/>
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="MW_H2O" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -485,20 +485,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K96"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:K95"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="4" max="4" width="17.36328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.36328125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.81640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.90625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.36328125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.81640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="9.7265625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -533,7 +533,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -568,7 +568,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -603,7 +603,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -638,7 +638,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>4</v>
       </c>
@@ -673,7 +673,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>5</v>
       </c>
@@ -708,7 +708,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>6</v>
       </c>
@@ -743,7 +743,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>7</v>
       </c>
@@ -778,7 +778,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>8</v>
       </c>
@@ -813,7 +813,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>9</v>
       </c>
@@ -848,7 +848,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>10</v>
       </c>
@@ -883,7 +883,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>10</v>
       </c>
@@ -918,7 +918,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>11</v>
       </c>
@@ -953,7 +953,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <v>12</v>
       </c>
@@ -988,7 +988,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
         <v>12</v>
       </c>
@@ -1023,7 +1023,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
         <v>12</v>
       </c>
@@ -1058,7 +1058,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
         <v>12</v>
       </c>
@@ -1093,7 +1093,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
         <v>13</v>
       </c>
@@ -1128,7 +1128,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
         <v>14</v>
       </c>
@@ -1163,7 +1163,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
         <v>15</v>
       </c>
@@ -1198,7 +1198,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
         <v>16</v>
       </c>
@@ -1233,7 +1233,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
         <v>17</v>
       </c>
@@ -1268,7 +1268,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
         <v>18</v>
       </c>
@@ -1303,7 +1303,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" s="1">
         <v>19</v>
       </c>
@@ -1338,7 +1338,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" s="1">
         <v>19</v>
       </c>
@@ -1373,7 +1373,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" s="1">
         <v>20</v>
       </c>
@@ -1408,7 +1408,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" s="1">
         <v>21</v>
       </c>
@@ -1443,7 +1443,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" s="1">
         <v>22</v>
       </c>
@@ -1478,7 +1478,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" s="1">
         <v>23</v>
       </c>
@@ -1513,7 +1513,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" s="1">
         <v>23</v>
       </c>
@@ -1548,7 +1548,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" s="1">
         <v>23</v>
       </c>
@@ -1583,7 +1583,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" s="1">
         <v>24</v>
       </c>
@@ -1618,7 +1618,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" s="1">
         <v>25</v>
       </c>
@@ -1653,7 +1653,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" s="1">
         <v>26</v>
       </c>
@@ -1688,7 +1688,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" s="1">
         <v>26</v>
       </c>
@@ -1723,7 +1723,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36" s="1">
         <v>27</v>
       </c>
@@ -1758,7 +1758,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" s="1">
         <v>27</v>
       </c>
@@ -1793,7 +1793,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" s="1">
         <v>27</v>
       </c>
@@ -1828,7 +1828,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" s="1">
         <v>28</v>
       </c>
@@ -1863,7 +1863,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40" s="1">
         <v>29</v>
       </c>
@@ -1898,7 +1898,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" s="1">
         <v>29</v>
       </c>
@@ -1933,7 +1933,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" s="1">
         <v>30</v>
       </c>
@@ -1968,7 +1968,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" s="1">
         <v>30</v>
       </c>
@@ -2003,7 +2003,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44" s="1">
         <v>31</v>
       </c>
@@ -2038,7 +2038,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" s="1">
         <v>32</v>
       </c>
@@ -2073,7 +2073,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A46" s="1">
         <v>33</v>
       </c>
@@ -2108,7 +2108,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A47" s="1">
         <v>34</v>
       </c>
@@ -2143,7 +2143,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" s="1">
         <v>34</v>
       </c>
@@ -2178,7 +2178,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A49" s="1">
         <v>35</v>
       </c>
@@ -2213,7 +2213,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A50" s="1">
         <v>35</v>
       </c>
@@ -2248,7 +2248,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A51" s="1">
         <v>35</v>
       </c>
@@ -2283,7 +2283,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A52" s="1">
         <v>36</v>
       </c>
@@ -2318,7 +2318,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53" s="1">
         <v>37</v>
       </c>
@@ -2353,7 +2353,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A54" s="1">
         <v>37</v>
       </c>
@@ -2388,7 +2388,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A55" s="1">
         <v>37</v>
       </c>
@@ -2423,7 +2423,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A56" s="1">
         <v>38</v>
       </c>
@@ -2458,7 +2458,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57" s="1">
         <v>39</v>
       </c>
@@ -2493,7 +2493,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A58" s="1">
         <v>39</v>
       </c>
@@ -2528,7 +2528,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A59" s="1">
         <v>40</v>
       </c>
@@ -2563,7 +2563,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A60" s="1">
         <v>41</v>
       </c>
@@ -2598,7 +2598,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A61" s="1">
         <v>42</v>
       </c>
@@ -2633,7 +2633,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A62" s="1">
         <v>42</v>
       </c>
@@ -2668,7 +2668,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A63" s="1">
         <v>43</v>
       </c>
@@ -2703,7 +2703,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A64" s="1">
         <v>44</v>
       </c>
@@ -2738,7 +2738,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="65" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A65" s="1">
         <v>44</v>
       </c>
@@ -2773,7 +2773,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="66" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A66" s="1">
         <v>45</v>
       </c>
@@ -2808,7 +2808,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="67" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A67" s="1">
         <v>46</v>
       </c>
@@ -2843,7 +2843,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="68" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A68" s="1">
         <v>47</v>
       </c>
@@ -2878,7 +2878,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="69" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A69" s="1">
         <v>47</v>
       </c>
@@ -2913,7 +2913,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="70" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A70" s="1">
         <v>47</v>
       </c>
@@ -2948,7 +2948,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="71" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A71" s="1">
         <v>47</v>
       </c>
@@ -2983,7 +2983,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="72" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A72" s="1">
         <v>47</v>
       </c>
@@ -3018,7 +3018,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="73" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A73" s="1">
         <v>47</v>
       </c>
@@ -3053,7 +3053,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="74" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A74" s="1">
         <v>47</v>
       </c>
@@ -3088,7 +3088,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="75" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A75" s="1">
         <v>47</v>
       </c>
@@ -3123,7 +3123,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="76" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A76" s="1">
         <v>47</v>
       </c>
@@ -3158,7 +3158,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="77" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A77" s="1">
         <v>48</v>
       </c>
@@ -3193,7 +3193,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="78" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A78" s="1">
         <v>48</v>
       </c>
@@ -3228,7 +3228,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="79" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A79" s="1">
         <v>49</v>
       </c>
@@ -3263,7 +3263,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="80" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A80" s="1">
         <v>49</v>
       </c>
@@ -3298,7 +3298,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="81" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A81" s="1">
         <v>49</v>
       </c>
@@ -3333,7 +3333,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="82" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A82" s="1">
         <v>50</v>
       </c>
@@ -3368,7 +3368,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="83" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A83" s="1">
         <v>50</v>
       </c>
@@ -3403,7 +3403,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="84" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A84" s="1">
         <v>50</v>
       </c>
@@ -3438,7 +3438,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="85" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A85" s="1">
         <v>51</v>
       </c>
@@ -3473,7 +3473,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="86" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A86" s="1">
         <v>52</v>
       </c>
@@ -3508,7 +3508,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="87" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A87" s="1">
         <v>53</v>
       </c>
@@ -3543,7 +3543,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="88" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A88" s="1">
         <v>54</v>
       </c>
@@ -3578,7 +3578,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="89" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A89" s="1">
         <v>55</v>
       </c>
@@ -3613,7 +3613,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="90" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A90" s="1">
         <v>55</v>
       </c>
@@ -3648,7 +3648,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="91" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A91" s="1">
         <v>55</v>
       </c>
@@ -3671,10 +3671,10 @@
         <v>907.96692115791996</v>
       </c>
       <c r="H91" s="3">
-        <v>618.97794743861323</v>
+        <v>622.77945806023581</v>
       </c>
       <c r="I91" s="3">
-        <v>329.98897371930673</v>
+        <v>331.88972903011791</v>
       </c>
       <c r="J91" s="3">
         <v>275.98897371930661</v>
@@ -3683,53 +3683,53 @@
         <v>18</v>
       </c>
     </row>
-    <row r="92" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A92" s="1">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B92" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C92" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D92" s="3">
-        <v>319.88972903011791</v>
+        <v>307.11144247140209</v>
       </c>
       <c r="E92" s="3">
         <v>92.09</v>
       </c>
       <c r="F92" s="3">
-        <v>46.07</v>
+        <v>32.04</v>
       </c>
       <c r="G92" s="3">
-        <v>913.6691870903536</v>
+        <v>917.33432741420654</v>
       </c>
       <c r="H92" s="3">
-        <v>622.77945806023581</v>
+        <v>625.22288494280428</v>
       </c>
       <c r="I92" s="3">
-        <v>331.88972903011791</v>
+        <v>333.11144247140209</v>
       </c>
       <c r="J92" s="3">
-        <v>277.88972903011791</v>
+        <v>279.11144247140209</v>
       </c>
       <c r="K92" s="1">
         <v>18</v>
       </c>
     </row>
-    <row r="93" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A93" s="1">
         <v>56</v>
       </c>
       <c r="B93" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C93" s="1">
         <v>1</v>
       </c>
       <c r="D93" s="3">
-        <v>307.11144247140209</v>
+        <v>306.32372747868811</v>
       </c>
       <c r="E93" s="3">
         <v>92.09</v>
@@ -3738,33 +3738,33 @@
         <v>32.04</v>
       </c>
       <c r="G93" s="3">
-        <v>917.33432741420654</v>
+        <v>914.9711824360644</v>
       </c>
       <c r="H93" s="3">
-        <v>625.22288494280428</v>
+        <v>623.64745495737623</v>
       </c>
       <c r="I93" s="3">
-        <v>333.11144247140209</v>
+        <v>332.32372747868811</v>
       </c>
       <c r="J93" s="3">
-        <v>279.11144247140209</v>
+        <v>278.32372747868811</v>
       </c>
       <c r="K93" s="1">
         <v>18</v>
       </c>
     </row>
-    <row r="94" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A94" s="1">
         <v>56</v>
       </c>
       <c r="B94" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C94" s="1">
         <v>1</v>
       </c>
       <c r="D94" s="3">
-        <v>306.32372747868811</v>
+        <v>305.5376248629949</v>
       </c>
       <c r="E94" s="3">
         <v>92.09</v>
@@ -3773,88 +3773,53 @@
         <v>32.04</v>
       </c>
       <c r="G94" s="3">
-        <v>914.9711824360644</v>
+        <v>912.61287458898482</v>
       </c>
       <c r="H94" s="3">
-        <v>623.64745495737623</v>
+        <v>622.07524972598981</v>
       </c>
       <c r="I94" s="3">
-        <v>332.32372747868811</v>
+        <v>331.5376248629949</v>
       </c>
       <c r="J94" s="3">
-        <v>278.32372747868811</v>
+        <v>277.5376248629949</v>
       </c>
       <c r="K94" s="1">
         <v>18</v>
       </c>
     </row>
-    <row r="95" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A95" s="1">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B95" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C95" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D95" s="3">
-        <v>305.5376248629949</v>
+        <v>245.61189439391251</v>
       </c>
       <c r="E95" s="3">
         <v>92.09</v>
       </c>
       <c r="F95" s="3">
-        <v>32.04</v>
+        <v>46.07</v>
       </c>
       <c r="G95" s="3">
-        <v>912.61287458898482</v>
+        <v>690.83568318173752</v>
       </c>
       <c r="H95" s="3">
-        <v>622.07524972598981</v>
+        <v>474.22378878782501</v>
       </c>
       <c r="I95" s="3">
-        <v>331.5376248629949</v>
+        <v>257.61189439391251</v>
       </c>
       <c r="J95" s="3">
-        <v>277.5376248629949</v>
+        <v>203.61189439391251</v>
       </c>
       <c r="K95" s="1">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="96" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A96" s="1">
-        <v>57</v>
-      </c>
-      <c r="B96" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C96" s="1">
-        <v>2</v>
-      </c>
-      <c r="D96" s="3">
-        <v>245.61189439391251</v>
-      </c>
-      <c r="E96" s="3">
-        <v>92.09</v>
-      </c>
-      <c r="F96" s="3">
-        <v>46.07</v>
-      </c>
-      <c r="G96" s="3">
-        <v>690.83568318173752</v>
-      </c>
-      <c r="H96" s="3">
-        <v>474.22378878782501</v>
-      </c>
-      <c r="I96" s="3">
-        <v>257.61189439391251</v>
-      </c>
-      <c r="J96" s="3">
-        <v>203.61189439391251</v>
-      </c>
-      <c r="K96" s="1">
         <v>18</v>
       </c>
     </row>

</xml_diff>